<commit_message>
Rellenar historia de instrumentos nuevos 2026-09-17
</commit_message>
<xml_diff>
--- a/historicos.xlsx
+++ b/historicos.xlsx
@@ -1994,6 +1994,9 @@
       <c r="HJ2" t="n">
         <v>105.35</v>
       </c>
+      <c r="HL2" t="n">
+        <v>100.6</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2493,6 +2496,9 @@
       <c r="HJ3" t="n">
         <v>106.75</v>
       </c>
+      <c r="HL3" t="n">
+        <v>102.75</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2995,6 +3001,9 @@
       <c r="HJ4" t="n">
         <v>106.15</v>
       </c>
+      <c r="HL4" t="n">
+        <v>103.2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3500,6 +3509,9 @@
       <c r="HJ5" t="n">
         <v>106.4</v>
       </c>
+      <c r="HL5" t="n">
+        <v>102.75</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4014,6 +4026,9 @@
       <c r="HJ6" t="n">
         <v>107</v>
       </c>
+      <c r="HL6" t="n">
+        <v>103</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4540,6 +4555,12 @@
       <c r="HJ7" t="n">
         <v>106.2</v>
       </c>
+      <c r="HL7" t="n">
+        <v>102.65</v>
+      </c>
+      <c r="HN7" t="n">
+        <v>103.8</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -5060,6 +5081,9 @@
       <c r="HJ8" t="n">
         <v>105.8</v>
       </c>
+      <c r="HL8" t="n">
+        <v>102.7</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -5586,6 +5610,9 @@
       <c r="HJ9" t="n">
         <v>106.2</v>
       </c>
+      <c r="HL9" t="n">
+        <v>102.9</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -6118,6 +6145,9 @@
       <c r="HJ10" t="n">
         <v>106.9</v>
       </c>
+      <c r="HL10" t="n">
+        <v>103.1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -6632,6 +6662,9 @@
       <c r="HJ11" t="n">
         <v>106.85</v>
       </c>
+      <c r="HL11" t="n">
+        <v>103.4</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -7143,6 +7176,9 @@
       <c r="HJ12" t="n">
         <v>106.3</v>
       </c>
+      <c r="HL12" t="n">
+        <v>103.05</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -7669,6 +7705,12 @@
       <c r="HJ13" t="n">
         <v>107.7</v>
       </c>
+      <c r="HL13" t="n">
+        <v>103.25</v>
+      </c>
+      <c r="HN13" t="n">
+        <v>103.55</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -8195,6 +8237,9 @@
       <c r="HJ14" t="n">
         <v>107.2</v>
       </c>
+      <c r="HL14" t="n">
+        <v>102.8</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -8715,6 +8760,9 @@
       <c r="HJ15" t="n">
         <v>108.5</v>
       </c>
+      <c r="HL15" t="n">
+        <v>103.2</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -9253,6 +9301,9 @@
       <c r="HJ16" t="n">
         <v>108.45</v>
       </c>
+      <c r="HL16" t="n">
+        <v>103.65</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -9788,6 +9839,9 @@
       <c r="HJ17" t="n">
         <v>107.5</v>
       </c>
+      <c r="HL17" t="n">
+        <v>103.15</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -10323,6 +10377,9 @@
       <c r="HJ18" t="n">
         <v>107.15</v>
       </c>
+      <c r="HL18" t="n">
+        <v>103.75</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -10858,6 +10915,9 @@
       <c r="HJ19" t="n">
         <v>106.9</v>
       </c>
+      <c r="HL19" t="n">
+        <v>103.2</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -11393,6 +11453,9 @@
       <c r="HJ20" t="n">
         <v>107.2</v>
       </c>
+      <c r="HL20" t="n">
+        <v>103.5</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -11931,6 +11994,12 @@
       <c r="HJ21" t="n">
         <v>106.9</v>
       </c>
+      <c r="HL21" t="n">
+        <v>104</v>
+      </c>
+      <c r="HN21" t="n">
+        <v>103.7</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -12484,6 +12553,12 @@
       <c r="HJ22" t="n">
         <v>107.7</v>
       </c>
+      <c r="HL22" t="n">
+        <v>103.2</v>
+      </c>
+      <c r="HN22" t="n">
+        <v>105.95</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -13028,6 +13103,9 @@
       <c r="HJ23" t="n">
         <v>107.75</v>
       </c>
+      <c r="HL23" t="n">
+        <v>103.1</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -13575,6 +13653,12 @@
       <c r="HJ24" t="n">
         <v>107.8</v>
       </c>
+      <c r="HL24" t="n">
+        <v>103.5</v>
+      </c>
+      <c r="HN24" t="n">
+        <v>106.4</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -14119,6 +14203,9 @@
       <c r="HJ25" t="n">
         <v>108.85</v>
       </c>
+      <c r="HL25" t="n">
+        <v>103.7</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -14654,6 +14741,9 @@
       <c r="HJ26" t="n">
         <v>107.75</v>
       </c>
+      <c r="HL26" t="n">
+        <v>104</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -15195,6 +15285,12 @@
       <c r="HJ27" t="n">
         <v>108.35</v>
       </c>
+      <c r="HL27" t="n">
+        <v>103.3</v>
+      </c>
+      <c r="HN27" t="n">
+        <v>106.35</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -15739,6 +15835,12 @@
       <c r="HJ28" t="n">
         <v>107.9</v>
       </c>
+      <c r="HL28" t="n">
+        <v>103.25</v>
+      </c>
+      <c r="HN28" t="n">
+        <v>106.15</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -16292,6 +16394,12 @@
       <c r="HJ29" t="n">
         <v>108.6</v>
       </c>
+      <c r="HL29" t="n">
+        <v>103.05</v>
+      </c>
+      <c r="HN29" t="n">
+        <v>106.95</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -16842,6 +16950,9 @@
       <c r="HJ30" t="n">
         <v>107.5</v>
       </c>
+      <c r="HL30" t="n">
+        <v>103.5</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -17401,6 +17512,12 @@
       <c r="HJ31" t="n">
         <v>107.2</v>
       </c>
+      <c r="HL31" t="n">
+        <v>104.05</v>
+      </c>
+      <c r="HN31" t="n">
+        <v>106</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -17951,6 +18068,12 @@
       <c r="HJ32" t="n">
         <v>107.4</v>
       </c>
+      <c r="HL32" t="n">
+        <v>104.1</v>
+      </c>
+      <c r="HN32" t="n">
+        <v>106.75</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -18507,6 +18630,9 @@
       <c r="HJ33" t="n">
         <v>107.25</v>
       </c>
+      <c r="HL33" t="n">
+        <v>104.85</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -18994,6 +19120,9 @@
       <c r="HJ34" t="n">
         <v>107.5</v>
       </c>
+      <c r="HL34" t="n">
+        <v>104.95</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -19556,6 +19685,12 @@
       <c r="HJ35" t="n">
         <v>107.45</v>
       </c>
+      <c r="HL35" t="n">
+        <v>104.05</v>
+      </c>
+      <c r="HN35" t="n">
+        <v>106.4</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -20115,6 +20250,12 @@
       <c r="HJ36" t="n">
         <v>107.7</v>
       </c>
+      <c r="HL36" t="n">
+        <v>103.8</v>
+      </c>
+      <c r="HN36" t="n">
+        <v>105.25</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -20674,6 +20815,12 @@
       <c r="HJ37" t="n">
         <v>108</v>
       </c>
+      <c r="HL37" t="n">
+        <v>103.9</v>
+      </c>
+      <c r="HN37" t="n">
+        <v>105.5</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -21236,6 +21383,12 @@
       <c r="HJ38" t="n">
         <v>108.1</v>
       </c>
+      <c r="HL38" t="n">
+        <v>104.05</v>
+      </c>
+      <c r="HN38" t="n">
+        <v>105.8</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -21813,6 +21966,12 @@
       <c r="HJ39" t="n">
         <v>108.4</v>
       </c>
+      <c r="HL39" t="n">
+        <v>103.85</v>
+      </c>
+      <c r="HN39" t="n">
+        <v>107</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -22375,6 +22534,12 @@
       <c r="HJ40" t="n">
         <v>108.1</v>
       </c>
+      <c r="HL40" t="n">
+        <v>104.4</v>
+      </c>
+      <c r="HN40" t="n">
+        <v>107</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -22937,6 +23102,12 @@
       <c r="HJ41" t="n">
         <v>108.35</v>
       </c>
+      <c r="HL41" t="n">
+        <v>103.5</v>
+      </c>
+      <c r="HN41" t="n">
+        <v>107</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -23502,6 +23673,12 @@
       <c r="HJ42" t="n">
         <v>106.5</v>
       </c>
+      <c r="HL42" t="n">
+        <v>104.5</v>
+      </c>
+      <c r="HN42" t="n">
+        <v>106.8</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -24064,6 +24241,12 @@
       <c r="HJ43" t="n">
         <v>107.4</v>
       </c>
+      <c r="HL43" t="n">
+        <v>104.5</v>
+      </c>
+      <c r="HN43" t="n">
+        <v>107</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -24644,6 +24827,12 @@
       <c r="HJ44" t="n">
         <v>106.3</v>
       </c>
+      <c r="HL44" t="n">
+        <v>103.75</v>
+      </c>
+      <c r="HN44" t="n">
+        <v>104.85</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -25221,6 +25410,12 @@
       <c r="HJ45" t="n">
         <v>105.2</v>
       </c>
+      <c r="HL45" t="n">
+        <v>104</v>
+      </c>
+      <c r="HN45" t="n">
+        <v>106.5</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -25798,6 +25993,12 @@
       <c r="HJ46" t="n">
         <v>106.3</v>
       </c>
+      <c r="HL46" t="n">
+        <v>104.45</v>
+      </c>
+      <c r="HO46" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -26372,6 +26573,15 @@
       <c r="HJ47" t="n">
         <v>105.4</v>
       </c>
+      <c r="HL47" t="n">
+        <v>104.1</v>
+      </c>
+      <c r="HN47" t="n">
+        <v>106.45</v>
+      </c>
+      <c r="HO47" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="n">
@@ -26932,6 +27142,12 @@
       <c r="HJ48" t="n">
         <v>104.9</v>
       </c>
+      <c r="HL48" t="n">
+        <v>104.45</v>
+      </c>
+      <c r="HO48" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="n">
@@ -27500,6 +27716,15 @@
       </c>
       <c r="HJ49" t="n">
         <v>105.05</v>
+      </c>
+      <c r="HL49" t="n">
+        <v>104.35</v>
+      </c>
+      <c r="HN49" t="n">
+        <v>108</v>
+      </c>
+      <c r="HO49" t="n">
+        <v>103</v>
       </c>
     </row>
     <row r="50">
@@ -28090,6 +28315,9 @@
       <c r="HJ50" t="n">
         <v>105.9</v>
       </c>
+      <c r="HL50" t="n">
+        <v>104.15</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -28670,6 +28898,9 @@
       <c r="HJ51" t="n">
         <v>105.9</v>
       </c>
+      <c r="HL51" t="n">
+        <v>104.5</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -29250,6 +29481,9 @@
       <c r="HJ52" t="n">
         <v>105.75</v>
       </c>
+      <c r="HL52" t="n">
+        <v>104.1</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="n">
@@ -29834,6 +30068,12 @@
       <c r="HJ53" t="n">
         <v>105.4</v>
       </c>
+      <c r="HL53" t="n">
+        <v>104.9</v>
+      </c>
+      <c r="HN53" t="n">
+        <v>108.4</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="n">
@@ -30417,6 +30657,12 @@
       </c>
       <c r="HJ54" t="n">
         <v>106.65</v>
+      </c>
+      <c r="HL54" t="n">
+        <v>104.8</v>
+      </c>
+      <c r="HN54" t="n">
+        <v>108.4</v>
       </c>
     </row>
     <row r="55">
@@ -31001,6 +31247,12 @@
       <c r="HJ55" t="n">
         <v>105.8</v>
       </c>
+      <c r="HL55" t="n">
+        <v>104</v>
+      </c>
+      <c r="HN55" t="n">
+        <v>108</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -31590,6 +31842,12 @@
       <c r="HJ56" t="n">
         <v>105.45</v>
       </c>
+      <c r="HL56" t="n">
+        <v>104</v>
+      </c>
+      <c r="HN56" t="n">
+        <v>108</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -32170,6 +32428,9 @@
       <c r="HJ57" t="n">
         <v>104.8</v>
       </c>
+      <c r="HL57" t="n">
+        <v>104.55</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -32750,6 +33011,12 @@
       <c r="HJ58" t="n">
         <v>105.7</v>
       </c>
+      <c r="HL58" t="n">
+        <v>103.75</v>
+      </c>
+      <c r="HN58" t="n">
+        <v>108</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -33339,6 +33606,12 @@
       <c r="HJ59" t="n">
         <v>105.4</v>
       </c>
+      <c r="HL59" t="n">
+        <v>104.8</v>
+      </c>
+      <c r="HN59" t="n">
+        <v>106.95</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -33928,6 +34201,9 @@
       <c r="HJ60" t="n">
         <v>105.7</v>
       </c>
+      <c r="HL60" t="n">
+        <v>104</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -34520,6 +34796,12 @@
       <c r="HJ61" t="n">
         <v>105</v>
       </c>
+      <c r="HL61" t="n">
+        <v>104.35</v>
+      </c>
+      <c r="HN61" t="n">
+        <v>107</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -35112,6 +35394,12 @@
       <c r="HJ62" t="n">
         <v>104.7</v>
       </c>
+      <c r="HL62" t="n">
+        <v>103.9</v>
+      </c>
+      <c r="HN62" t="n">
+        <v>107</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -35704,6 +35992,9 @@
       <c r="HJ63" t="n">
         <v>104.7</v>
       </c>
+      <c r="HL63" t="n">
+        <v>104.4</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -36251,6 +36542,12 @@
       <c r="HJ64" t="n">
         <v>104.5</v>
       </c>
+      <c r="HL64" t="n">
+        <v>103.6</v>
+      </c>
+      <c r="HN64" t="n">
+        <v>107.2</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -36849,6 +37146,12 @@
       <c r="HJ65" t="n">
         <v>104.1</v>
       </c>
+      <c r="HL65" t="n">
+        <v>104</v>
+      </c>
+      <c r="HN65" t="n">
+        <v>107</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -37438,6 +37741,9 @@
       <c r="HJ66" t="n">
         <v>104.35</v>
       </c>
+      <c r="HL66" t="n">
+        <v>103.4</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -38033,6 +38339,9 @@
       <c r="HJ67" t="n">
         <v>104</v>
       </c>
+      <c r="HL67" t="n">
+        <v>104</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -38610,6 +38919,9 @@
       <c r="HJ68" t="n">
         <v>104.9</v>
       </c>
+      <c r="HL68" t="n">
+        <v>103.9</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -39193,6 +39505,9 @@
       <c r="HJ69" t="n">
         <v>104.95</v>
       </c>
+      <c r="HL69" t="n">
+        <v>104</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -39776,6 +40091,9 @@
       <c r="HJ70" t="n">
         <v>104.9</v>
       </c>
+      <c r="HL70" t="n">
+        <v>104</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -40362,6 +40680,9 @@
       <c r="HJ71" t="n">
         <v>105</v>
       </c>
+      <c r="HL71" t="n">
+        <v>103.95</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -40948,6 +41269,15 @@
       <c r="HJ72" t="n">
         <v>105.55</v>
       </c>
+      <c r="HL72" t="n">
+        <v>103.85</v>
+      </c>
+      <c r="HN72" t="n">
+        <v>107</v>
+      </c>
+      <c r="HO72" t="n">
+        <v>100.3</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -41534,6 +41864,9 @@
       <c r="HJ73" t="n">
         <v>105.5</v>
       </c>
+      <c r="HL73" t="n">
+        <v>103.7</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -42120,6 +42453,12 @@
       <c r="HJ74" t="n">
         <v>105.3</v>
       </c>
+      <c r="HL74" t="n">
+        <v>103.75</v>
+      </c>
+      <c r="HM74" t="n">
+        <v>100.5</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -42709,6 +43048,15 @@
       <c r="HJ75" t="n">
         <v>104.6</v>
       </c>
+      <c r="HL75" t="n">
+        <v>103.45</v>
+      </c>
+      <c r="HM75" t="n">
+        <v>100.55</v>
+      </c>
+      <c r="HN75" t="n">
+        <v>103.95</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -43295,6 +43643,15 @@
       <c r="HJ76" t="n">
         <v>104.3</v>
       </c>
+      <c r="HL76" t="n">
+        <v>103.8</v>
+      </c>
+      <c r="HM76" t="n">
+        <v>101.5</v>
+      </c>
+      <c r="HN76" t="n">
+        <v>105.8</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -43884,6 +44241,15 @@
       <c r="HJ77" t="n">
         <v>104.8</v>
       </c>
+      <c r="HL77" t="n">
+        <v>104.4</v>
+      </c>
+      <c r="HM77" t="n">
+        <v>100.5</v>
+      </c>
+      <c r="HN77" t="n">
+        <v>103.2</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -44470,6 +44836,18 @@
       <c r="HJ78" t="n">
         <v>104.9</v>
       </c>
+      <c r="HL78" t="n">
+        <v>104.5</v>
+      </c>
+      <c r="HM78" t="n">
+        <v>101</v>
+      </c>
+      <c r="HN78" t="n">
+        <v>105</v>
+      </c>
+      <c r="HO78" t="n">
+        <v>100.5</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -45059,6 +45437,18 @@
       <c r="HJ79" t="n">
         <v>105.35</v>
       </c>
+      <c r="HL79" t="n">
+        <v>104.65</v>
+      </c>
+      <c r="HM79" t="n">
+        <v>100.25</v>
+      </c>
+      <c r="HN79" t="n">
+        <v>104.3</v>
+      </c>
+      <c r="HO79" t="n">
+        <v>100.5</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">

</xml_diff>